<commit_message>
MoSe2 pattern and file path changes
</commit_message>
<xml_diff>
--- a/EQE/Plots/Processed data from Results table.xlsx
+++ b/EQE/Plots/Processed data from Results table.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_200Sb_25Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_200Sb_25Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -5617,7 +5617,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -5773,7 +5773,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -6163,7 +6163,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_300Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_300Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400deg_400Sb_35Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400deg_400Sb_35Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -7361,7 +7361,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -7673,7 +7673,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -8063,7 +8063,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>C:/Users/jp_ol/OneDrive/Ambiente de Trabalho/TESE/Data_Analysis/data/2nd Round/Corrected/Mo_400Sb_30Se_Results Table.txt</t>
+          <t>C:\Users\jp_ol\OneDrive\Ambiente de Trabalho\TESE\Data_Analysis\data\2nd Round\Corrected\Mo_400Sb_30Se_Results Table.txt</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">

</xml_diff>